<commit_message>
20250818 - update of rmarkdown
update of rmarkdown with the new data
</commit_message>
<xml_diff>
--- a/data_u1/data_2025-08-15_LSR3_H.xlsx
+++ b/data_u1/data_2025-08-15_LSR3_H.xlsx
@@ -1133,7 +1133,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>70.7</t>
+          <t>70.400000000000006</t>
         </is>
       </c>
       <c r="N2">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>70.7</t>
+          <t>71.8</t>
         </is>
       </c>
       <c r="N3">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>30.3</t>
+          <t>30</t>
         </is>
       </c>
       <c r="N4">
@@ -2228,7 +2228,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>30.3</t>
+          <t>30.6</t>
         </is>
       </c>
       <c r="N5">
@@ -2821,7 +2821,7 @@
         <v>-5.7</v>
       </c>
       <c r="AW6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AX6" t="inlineStr">
         <is>
@@ -2856,7 +2856,7 @@
         <v>-5.5</v>
       </c>
       <c r="BF6">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="BG6" t="inlineStr">
         <is>
@@ -3162,7 +3162,7 @@
         <v>-7</v>
       </c>
       <c r="AW7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AX7" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         <v>-7.3</v>
       </c>
       <c r="BF7">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="BG7" t="inlineStr">
         <is>
@@ -3412,7 +3412,7 @@
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -3503,7 +3503,7 @@
         <v>-6.4</v>
       </c>
       <c r="AW8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AX8" t="inlineStr">
         <is>
@@ -3538,7 +3538,7 @@
         <v>-6.2</v>
       </c>
       <c r="BF8">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="BG8" t="inlineStr">
         <is>
@@ -3653,7 +3653,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NCT04072354 (2019, adolescent)</t>
+          <t>NCT04072354 (2019):adolescents</t>
         </is>
       </c>
       <c r="C9">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="EM9" t="inlineStr">
         <is>
-          <t>NCT04072354 (2019, adolescent) - ulotaront</t>
+          <t>NCT04072354 (2019):adolescents - ulotaront</t>
         </is>
       </c>
       <c r="EN9">
@@ -3884,7 +3884,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>NCT04072354 (2019, adolescent)</t>
+          <t>NCT04072354 (2019):adolescents</t>
         </is>
       </c>
       <c r="C10">
@@ -4100,7 +4100,7 @@
       </c>
       <c r="EM10" t="inlineStr">
         <is>
-          <t>NCT04072354 (2019, adolescent) - ulotaront</t>
+          <t>NCT04072354 (2019):adolescents - ulotaront</t>
         </is>
       </c>
       <c r="EN10">
@@ -4115,7 +4115,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NCT04072354 (2019, adolescent)</t>
+          <t>NCT04072354 (2019):adolescents</t>
         </is>
       </c>
       <c r="C11">
@@ -4331,7 +4331,7 @@
       </c>
       <c r="EM11" t="inlineStr">
         <is>
-          <t>NCT04072354 (2019, adolescent) - ulotaront</t>
+          <t>NCT04072354 (2019):adolescents - ulotaront</t>
         </is>
       </c>
       <c r="EN11">
@@ -4537,7 +4537,7 @@
         <v>-5.2</v>
       </c>
       <c r="AW12">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AX12" t="inlineStr">
         <is>
@@ -4572,7 +4572,7 @@
         <v>-6</v>
       </c>
       <c r="BF12">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="BG12" t="inlineStr">
         <is>
@@ -4860,7 +4860,7 @@
         <v>-5.5</v>
       </c>
       <c r="AW13">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AX13" t="inlineStr">
         <is>
@@ -4895,7 +4895,7 @@
         <v>-6.4</v>
       </c>
       <c r="BF13">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="BG13" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
         <v>-4.6</v>
       </c>
       <c r="AW14">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AX14" t="inlineStr">
         <is>
@@ -5218,7 +5218,7 @@
         <v>-4.5</v>
       </c>
       <c r="BF14">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="BG14" t="inlineStr">
         <is>
@@ -5359,7 +5359,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>33.1</t>
+          <t>33.200000000000003</t>
         </is>
       </c>
       <c r="N15">
@@ -5717,7 +5717,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>33.1</t>
+          <t>34</t>
         </is>
       </c>
       <c r="N16">
@@ -6075,7 +6075,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>33.1</t>
+          <t>32.299999999999997</t>
         </is>
       </c>
       <c r="N17">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>33.1</t>
+          <t>32.9</t>
         </is>
       </c>
       <c r="N18">
@@ -8482,7 +8482,7 @@
         </is>
       </c>
       <c r="S30">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="T30">
         <v>201</v>
@@ -8539,7 +8539,7 @@
       </c>
       <c r="AE30" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Some concerns</t>
         </is>
       </c>
       <c r="AF30" t="inlineStr">
@@ -8554,7 +8554,7 @@
       </c>
       <c r="AH30" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="AI30" t="inlineStr">
@@ -8648,12 +8648,12 @@
       </c>
       <c r="CZ30" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="DA30" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="DB30">
@@ -8669,7 +8669,7 @@
         <v>201</v>
       </c>
       <c r="DF30">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="DG30">
         <v>201</v>
@@ -8717,7 +8717,7 @@
         <v>201</v>
       </c>
       <c r="EF30">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="EG30">
         <v>201</v>
@@ -8813,7 +8813,7 @@
         </is>
       </c>
       <c r="S31">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="T31">
         <v>102</v>
@@ -8870,7 +8870,7 @@
       </c>
       <c r="AE31" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Some concerns</t>
         </is>
       </c>
       <c r="AF31" t="inlineStr">
@@ -8885,7 +8885,7 @@
       </c>
       <c r="AH31" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="AI31" t="inlineStr">
@@ -8979,12 +8979,12 @@
       </c>
       <c r="CZ31" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="DA31" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="DB31">
@@ -9743,7 +9743,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>NCT03669640 (2018, addon)</t>
+          <t>NCT03669640 (2018):addon</t>
         </is>
       </c>
       <c r="C34">
@@ -10057,7 +10057,7 @@
       </c>
       <c r="EM34" t="inlineStr">
         <is>
-          <t>NCT03669640 (2018, addon) - ulotaront</t>
+          <t>NCT03669640 (2018):addon - ulotaront</t>
         </is>
       </c>
       <c r="EN34">
@@ -10072,7 +10072,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>NCT03669640 (2018, addon)</t>
+          <t>NCT03669640 (2018):addon</t>
         </is>
       </c>
       <c r="C35">
@@ -10386,7 +10386,7 @@
       </c>
       <c r="EM35" t="inlineStr">
         <is>
-          <t>NCT03669640 (2018, addon) - ulotaront</t>
+          <t>NCT03669640 (2018):addon - ulotaront</t>
         </is>
       </c>
       <c r="EN35">
@@ -10401,7 +10401,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>NCT03669640 (2018, addon)</t>
+          <t>NCT03669640 (2018):addon</t>
         </is>
       </c>
       <c r="C36">
@@ -10715,7 +10715,7 @@
       </c>
       <c r="EM36" t="inlineStr">
         <is>
-          <t>NCT03669640 (2018, addon) - ulotaront</t>
+          <t>NCT03669640 (2018):addon - ulotaront</t>
         </is>
       </c>
       <c r="EN36">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>NCT03669640 (2018, addon)</t>
+          <t>NCT03669640 (2018):addon</t>
         </is>
       </c>
       <c r="C37">
@@ -11044,7 +11044,7 @@
       </c>
       <c r="EM37" t="inlineStr">
         <is>
-          <t>NCT03669640 (2018, addon) - ulotaront</t>
+          <t>NCT03669640 (2018):addon - ulotaront</t>
         </is>
       </c>
       <c r="EN37">

</xml_diff>